<commit_message>
Updated default mission plan with 20 LEOP sequence samples & remark integration
</commit_message>
<xml_diff>
--- a/final_output/20260726_test.xlsx
+++ b/final_output/20260726_test.xlsx
@@ -36,7 +36,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -51,14 +51,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F9FF"/>
-        <bgColor rgb="00F2F9FF"/>
+        <fgColor rgb="00E8EAF6"/>
+        <bgColor rgb="00E8EAF6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFBF0"/>
-        <bgColor rgb="00FFFBF0"/>
+        <fgColor rgb="00E0F2F1"/>
+        <bgColor rgb="00E0F2F1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3E0"/>
+        <bgColor rgb="00FFF3E0"/>
       </patternFill>
     </fill>
   </fills>
@@ -74,11 +80,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -544,134 +551,136 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
+          <t>[1] First Contact (TM 확인
+Panel 전개
+TLE update)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Svalbard</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>NEONSAT-1A(67614)</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Pass 2</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-26 12:29:06</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-26 12:38:10</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>543.7</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>30.77</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Allocated</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
           <t>[1] First Contact (TM 확인 / Panel 전개 / TLE update)</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Svalbard</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>NEONSAT-1A(67614)</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Pass 2</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-26 12:29:06</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-26 12:38:10</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="n">
-        <v>543.7</v>
-      </c>
-      <c r="G3" s="3" t="n">
-        <v>30.77</v>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>King Sejong</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>NEONSAT-1(59587)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Pass 3</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-26 12:30:52</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-26 12:37:57</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>424.2</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>17.59</v>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Allocated</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>[1] First Contact (TM 확인 / Panel 전개 / TLE update)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>King Sejong</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>[2] Health check (EPS / AOCS / S-band 상태 점검)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Daejeon</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>NEONSAT-1(59587)</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Pass 3</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-26 12:30:52</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-26 12:37:57</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="n">
-        <v>424.2</v>
-      </c>
-      <c r="G4" s="2" t="n">
-        <v>17.59</v>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-26 13:11:13</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-26 13:16:48</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>335.3</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>11.08</v>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>Allocated</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>[2] Health check (EPS / AOCS / S-band 상태 점검)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Daejeon</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>NEONSAT-1(59587)</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Pass 3</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-26 13:11:13</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-26 13:16:48</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="n">
-        <v>335.3</v>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>11.08</v>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>Allocated</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>[3] Configuration check (Thermal / STX / FCS param 확인)</t>
         </is>
@@ -721,129 +730,129 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>King Sejong</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>NEONSAT-1(59587)</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>Pass 4</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>2026-07-26 14:02:21</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>2026-07-26 14:11:03</t>
         </is>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="F7" s="3" t="n">
         <v>522</v>
       </c>
-      <c r="G7" s="2" t="n">
+      <c r="G7" s="3" t="n">
         <v>87.02</v>
       </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>Bypassed</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Bypassed</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>[1차 지상 촬영] Blocked (GS King Sejong No DOWN)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Svalbard</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>NEONSAT-1A(67614)</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Pass 3</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>2026-07-26 14:03:59</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>2026-07-26 14:13:37</t>
         </is>
       </c>
-      <c r="F8" s="3" t="n">
+      <c r="F8" s="2" t="n">
         <v>577.8</v>
       </c>
-      <c r="G8" s="3" t="n">
+      <c r="G8" s="2" t="n">
         <v>63.5</v>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>Allocated</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>[2] Health check (EPS / AOCS / S-band 상태 점검)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Daejeon</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>NEONSAT-1(59587)</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Pass 4</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>2026-07-26 14:42:19</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>2026-07-26 14:50:26</t>
         </is>
       </c>
-      <c r="F9" s="2" t="n">
+      <c r="F9" s="4" t="n">
         <v>486.8</v>
       </c>
-      <c r="G9" s="2" t="n">
+      <c r="G9" s="4" t="n">
         <v>32.61</v>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>Allocated</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I9" s="4" t="inlineStr">
         <is>
           <t>[5] 1차 지상 촬영 (시나리오 등록 / 이미징 / 다운로드)</t>
         </is>
@@ -936,129 +945,129 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Daejeon</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>NEONSAT-1A(67614)</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>Pass 4</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>2026-07-26 15:25:14</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>2026-07-26 15:31:42</t>
         </is>
       </c>
-      <c r="F12" s="3" t="n">
+      <c r="F12" s="4" t="n">
         <v>387.8</v>
       </c>
-      <c r="G12" s="3" t="n">
+      <c r="G12" s="4" t="n">
         <v>12.21</v>
       </c>
-      <c r="H12" s="3" t="inlineStr">
-        <is>
-          <t>Bypassed</t>
-        </is>
-      </c>
-      <c r="I12" s="3" t="inlineStr">
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>Bypassed</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
         <is>
           <t>[X-band Key update] Blocked (El Low (12.21° &lt; 15.0°))</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>King Sejong</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>NEONSAT-1(59587)</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>Pass 5</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>2026-07-26 15:36:29</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E13" s="3" t="inlineStr">
         <is>
           <t>2026-07-26 15:43:22</t>
         </is>
       </c>
-      <c r="F13" s="2" t="n">
+      <c r="F13" s="3" t="n">
         <v>413.1</v>
       </c>
-      <c r="G13" s="2" t="n">
+      <c r="G13" s="3" t="n">
         <v>15.61</v>
       </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>Bypassed</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Bypassed</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
         <is>
           <t>[1차 Cal Maneuver] Blocked (GS King Sejong No BOTH)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Svalbard</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>NEONSAT-1A(67614)</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>Pass 4</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>2026-07-26 15:38:42</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>2026-07-26 15:48:20</t>
         </is>
       </c>
-      <c r="F14" s="3" t="n">
+      <c r="F14" s="2" t="n">
         <v>577.4</v>
       </c>
-      <c r="G14" s="3" t="n">
+      <c r="G14" s="2" t="n">
         <v>70.83</v>
       </c>
-      <c r="H14" s="3" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>Allocated</t>
         </is>
       </c>
-      <c r="I14" s="3" t="inlineStr">
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>[4] X-band Key update (X key update)</t>
         </is>
@@ -1151,86 +1160,86 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>Daejeon</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>NEONSAT-1A(67614)</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>Pass 5</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>2026-07-26 16:58:02</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>2026-07-26 17:07:15</t>
         </is>
       </c>
-      <c r="F17" s="3" t="n">
+      <c r="F17" s="4" t="n">
         <v>553.1</v>
       </c>
-      <c r="G17" s="3" t="n">
+      <c r="G17" s="4" t="n">
         <v>39.8</v>
       </c>
-      <c r="H17" s="3" t="inlineStr">
+      <c r="H17" s="4" t="inlineStr">
         <is>
           <t>Allocated</t>
         </is>
       </c>
-      <c r="I17" s="3" t="inlineStr">
+      <c r="I17" s="4" t="inlineStr">
         <is>
           <t>[5] 1차 지상 촬영 (시나리오 등록 / 이미징 / 다운로드)</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>Svalbard</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>NEONSAT-1A(67614)</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>Pass 5</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>2026-07-26 17:13:12</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>2026-07-26 17:22:38</t>
         </is>
       </c>
-      <c r="F18" s="3" t="n">
+      <c r="F18" s="2" t="n">
         <v>565.3</v>
       </c>
-      <c r="G18" s="3" t="n">
+      <c r="G18" s="2" t="n">
         <v>48.57</v>
       </c>
-      <c r="H18" s="3" t="inlineStr">
-        <is>
-          <t>Bypassed</t>
-        </is>
-      </c>
-      <c r="I18" s="3" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Bypassed</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>[1차 Cal Maneuver] Blocked (GS Svalbard No BOTH)</t>
         </is>
@@ -1323,43 +1332,43 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>Svalbard</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>NEONSAT-1A(67614)</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>Pass 6</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>2026-07-26 18:47:29</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>2026-07-26 18:56:51</t>
         </is>
       </c>
-      <c r="F21" s="3" t="n">
+      <c r="F21" s="2" t="n">
         <v>561.6</v>
       </c>
-      <c r="G21" s="3" t="n">
+      <c r="G21" s="2" t="n">
         <v>45.21</v>
       </c>
-      <c r="H21" s="3" t="inlineStr">
-        <is>
-          <t>Bypassed</t>
-        </is>
-      </c>
-      <c r="I21" s="3" t="inlineStr">
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Bypassed</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
         <is>
           <t>[1차 Cal Maneuver] Blocked (GS Svalbard No BOTH)</t>
         </is>
@@ -1409,43 +1418,43 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>Svalbard</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>NEONSAT-1A(67614)</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>Pass 7</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>2026-07-26 20:21:43</t>
         </is>
       </c>
-      <c r="E23" s="3" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>2026-07-26 20:31:14</t>
         </is>
       </c>
-      <c r="F23" s="3" t="n">
+      <c r="F23" s="2" t="n">
         <v>571.1</v>
       </c>
-      <c r="G23" s="3" t="n">
+      <c r="G23" s="2" t="n">
         <v>57.39</v>
       </c>
-      <c r="H23" s="3" t="inlineStr">
-        <is>
-          <t>Bypassed</t>
-        </is>
-      </c>
-      <c r="I23" s="3" t="inlineStr">
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Bypassed</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
         <is>
           <t>[1차 Cal Maneuver] Blocked (GS Svalbard No BOTH)</t>
         </is>
@@ -1495,43 +1504,43 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>Svalbard</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t>NEONSAT-1A(67614)</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="C25" s="2" t="inlineStr">
         <is>
           <t>Pass 8</t>
         </is>
       </c>
-      <c r="D25" s="3" t="inlineStr">
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>2026-07-26 21:56:12</t>
         </is>
       </c>
-      <c r="E25" s="3" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>2026-07-26 22:05:52</t>
         </is>
       </c>
-      <c r="F25" s="3" t="n">
+      <c r="F25" s="2" t="n">
         <v>579.4</v>
       </c>
-      <c r="G25" s="3" t="n">
+      <c r="G25" s="2" t="n">
         <v>85.79000000000001</v>
       </c>
-      <c r="H25" s="3" t="inlineStr">
-        <is>
-          <t>Bypassed</t>
-        </is>
-      </c>
-      <c r="I25" s="3" t="inlineStr">
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Bypassed</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
         <is>
           <t>[1차 Cal Maneuver] Blocked (GS Svalbard No BOTH)</t>
         </is>
@@ -1581,43 +1590,43 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>Svalbard</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>NEONSAT-1A(67614)</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr">
+      <c r="C27" s="2" t="inlineStr">
         <is>
           <t>Pass 9</t>
         </is>
       </c>
-      <c r="D27" s="3" t="inlineStr">
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>2026-07-26 23:31:17</t>
         </is>
       </c>
-      <c r="E27" s="3" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>2026-07-26 23:40:40</t>
         </is>
       </c>
-      <c r="F27" s="3" t="n">
+      <c r="F27" s="2" t="n">
         <v>563.6</v>
       </c>
-      <c r="G27" s="3" t="n">
+      <c r="G27" s="2" t="n">
         <v>42.64</v>
       </c>
-      <c r="H27" s="3" t="inlineStr">
-        <is>
-          <t>Bypassed</t>
-        </is>
-      </c>
-      <c r="I27" s="3" t="inlineStr">
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Bypassed</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
         <is>
           <t>[1차 Cal Maneuver] Blocked (GS Svalbard No BOTH)</t>
         </is>
@@ -1667,301 +1676,301 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="inlineStr">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>Svalbard</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>NEONSAT-1A(67614)</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr">
+      <c r="C29" s="2" t="inlineStr">
         <is>
           <t>Pass 10</t>
         </is>
       </c>
-      <c r="D29" s="3" t="inlineStr">
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>2026-07-27 01:07:14</t>
         </is>
       </c>
-      <c r="E29" s="3" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>2026-07-27 01:15:37</t>
         </is>
       </c>
-      <c r="F29" s="3" t="n">
+      <c r="F29" s="2" t="n">
         <v>503</v>
       </c>
-      <c r="G29" s="3" t="n">
+      <c r="G29" s="2" t="n">
         <v>21.37</v>
       </c>
-      <c r="H29" s="3" t="inlineStr">
-        <is>
-          <t>Bypassed</t>
-        </is>
-      </c>
-      <c r="I29" s="3" t="inlineStr">
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Bypassed</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
         <is>
           <t>[1차 Cal Maneuver] Blocked (GS Svalbard No BOTH)</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>Daejeon</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <t>NEONSAT-1(59587)</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="C30" s="4" t="inlineStr">
         <is>
           <t>Pass 12</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="D30" s="4" t="inlineStr">
         <is>
           <t>2026-07-27 02:06:36</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="E30" s="4" t="inlineStr">
         <is>
           <t>2026-07-27 02:13:18</t>
         </is>
       </c>
-      <c r="F30" s="2" t="n">
+      <c r="F30" s="4" t="n">
         <v>401.7</v>
       </c>
-      <c r="G30" s="2" t="n">
+      <c r="G30" s="4" t="n">
         <v>15.39</v>
       </c>
-      <c r="H30" s="2" t="inlineStr">
+      <c r="H30" s="4" t="inlineStr">
         <is>
           <t>Allocated</t>
         </is>
       </c>
-      <c r="I30" s="2" t="inlineStr">
+      <c r="I30" s="4" t="inlineStr">
         <is>
           <t>[6] 1차 Cal Maneuver (시나리오 등록 / Max logging / AOTM 다운)</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>Svalbard</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B31" s="2" t="inlineStr">
         <is>
           <t>NEONSAT-1A(67614)</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>Pass 11</t>
         </is>
       </c>
-      <c r="D31" s="3" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>2026-07-27 02:44:12</t>
         </is>
       </c>
-      <c r="E31" s="3" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>2026-07-27 02:50:36</t>
         </is>
       </c>
-      <c r="F31" s="3" t="n">
+      <c r="F31" s="2" t="n">
         <v>383.3</v>
       </c>
-      <c r="G31" s="3" t="n">
+      <c r="G31" s="2" t="n">
         <v>11.32</v>
       </c>
-      <c r="H31" s="3" t="inlineStr">
-        <is>
-          <t>Bypassed</t>
-        </is>
-      </c>
-      <c r="I31" s="3" t="inlineStr">
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Bypassed</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
         <is>
           <t>[1차 Cal Maneuver] Blocked (El Low (11.32° &lt; 15.0°), GS Svalbard No BOTH)</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>King Sejong</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="B32" s="3" t="inlineStr">
         <is>
           <t>NEONSAT-1(59587)</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
+      <c r="C32" s="3" t="inlineStr">
         <is>
           <t>Pass 12</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="D32" s="3" t="inlineStr">
         <is>
           <t>2026-07-27 02:46:00</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="E32" s="3" t="inlineStr">
         <is>
           <t>2026-07-27 02:53:42</t>
         </is>
       </c>
-      <c r="F32" s="2" t="n">
+      <c r="F32" s="3" t="n">
         <v>462.3</v>
       </c>
-      <c r="G32" s="2" t="n">
+      <c r="G32" s="3" t="n">
         <v>22.11</v>
       </c>
-      <c r="H32" s="2" t="inlineStr">
-        <is>
-          <t>Bypassed</t>
-        </is>
-      </c>
-      <c r="I32" s="2" t="inlineStr">
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>Bypassed</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="inlineStr">
         <is>
           <t>[2차 Cal Maneuver] Blocked (GS King Sejong No BOTH)</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>Daejeon</t>
         </is>
       </c>
-      <c r="B33" s="2" t="inlineStr">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>NEONSAT-1(59587)</t>
         </is>
       </c>
-      <c r="C33" s="2" t="inlineStr">
+      <c r="C33" s="4" t="inlineStr">
         <is>
           <t>Pass 13</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr">
+      <c r="D33" s="4" t="inlineStr">
         <is>
           <t>2026-07-27 03:38:53</t>
         </is>
       </c>
-      <c r="E33" s="2" t="inlineStr">
+      <c r="E33" s="4" t="inlineStr">
         <is>
           <t>2026-07-27 03:46:20</t>
         </is>
       </c>
-      <c r="F33" s="2" t="n">
+      <c r="F33" s="4" t="n">
         <v>446.6</v>
       </c>
-      <c r="G33" s="2" t="n">
+      <c r="G33" s="4" t="n">
         <v>22.07</v>
       </c>
-      <c r="H33" s="2" t="inlineStr">
+      <c r="H33" s="4" t="inlineStr">
         <is>
           <t>Allocated</t>
         </is>
       </c>
-      <c r="I33" s="2" t="inlineStr">
+      <c r="I33" s="4" t="inlineStr">
         <is>
           <t>[7] 2차 Cal Maneuver (시나리오 등록 / Max logging / AOTM 다운)</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="A34" s="3" t="inlineStr">
         <is>
           <t>King Sejong</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B34" s="3" t="inlineStr">
         <is>
           <t>NEONSAT-1(59587)</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr">
+      <c r="C34" s="3" t="inlineStr">
         <is>
           <t>Pass 13</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="D34" s="3" t="inlineStr">
         <is>
           <t>2026-07-27 04:18:33</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="E34" s="3" t="inlineStr">
         <is>
           <t>2026-07-27 04:27:11</t>
         </is>
       </c>
-      <c r="F34" s="2" t="n">
+      <c r="F34" s="3" t="n">
         <v>517.4</v>
       </c>
-      <c r="G34" s="2" t="n">
+      <c r="G34" s="3" t="n">
         <v>58.23</v>
       </c>
-      <c r="H34" s="2" t="inlineStr">
-        <is>
-          <t>Bypassed</t>
-        </is>
-      </c>
-      <c r="I34" s="2" t="inlineStr">
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>Bypassed</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
         <is>
           <t>[3차 Cal Maneuver] Blocked (GS King Sejong No BOTH)</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="3" t="inlineStr">
+      <c r="A35" s="4" t="inlineStr">
         <is>
           <t>Daejeon</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B35" s="4" t="inlineStr">
         <is>
           <t>NEONSAT-1A(67614)</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr">
+      <c r="C35" s="4" t="inlineStr">
         <is>
           <t>Pass 13</t>
         </is>
       </c>
-      <c r="D35" s="3" t="inlineStr">
+      <c r="D35" s="4" t="inlineStr">
         <is>
           <t>2026-07-27 04:35:42</t>
         </is>
       </c>
-      <c r="E35" s="3" t="inlineStr">
+      <c r="E35" s="4" t="inlineStr">
         <is>
           <t>2026-07-27 04:44:25</t>
         </is>
       </c>
-      <c r="F35" s="3" t="n">
+      <c r="F35" s="4" t="n">
         <v>522.6</v>
       </c>
-      <c r="G35" s="3" t="n">
+      <c r="G35" s="4" t="n">
         <v>25.53</v>
       </c>
-      <c r="H35" s="3" t="inlineStr">
+      <c r="H35" s="4" t="inlineStr">
         <is>
           <t>Allocated</t>
         </is>
       </c>
-      <c r="I35" s="3" t="inlineStr">
+      <c r="I35" s="4" t="inlineStr">
         <is>
           <t>[6] 1차 Cal Maneuver (시나리오 등록 / Max logging / AOTM 다운)</t>
         </is>
@@ -2011,86 +2020,86 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>King Sejong</t>
         </is>
       </c>
-      <c r="B37" s="2" t="inlineStr">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>NEONSAT-1(59587)</t>
         </is>
       </c>
-      <c r="C37" s="2" t="inlineStr">
+      <c r="C37" s="3" t="inlineStr">
         <is>
           <t>Pass 14</t>
         </is>
       </c>
-      <c r="D37" s="2" t="inlineStr">
+      <c r="D37" s="3" t="inlineStr">
         <is>
           <t>2026-07-27 05:51:47</t>
         </is>
       </c>
-      <c r="E37" s="2" t="inlineStr">
+      <c r="E37" s="3" t="inlineStr">
         <is>
           <t>2026-07-27 05:58:09</t>
         </is>
       </c>
-      <c r="F37" s="2" t="n">
+      <c r="F37" s="3" t="n">
         <v>381.3</v>
       </c>
-      <c r="G37" s="2" t="n">
+      <c r="G37" s="3" t="n">
         <v>13.59</v>
       </c>
-      <c r="H37" s="2" t="inlineStr">
-        <is>
-          <t>Bypassed</t>
-        </is>
-      </c>
-      <c r="I37" s="2" t="inlineStr">
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>Bypassed</t>
+        </is>
+      </c>
+      <c r="I37" s="3" t="inlineStr">
         <is>
           <t>[3차 Cal Maneuver] Blocked (El Low (13.59° &lt; 15.0°), GS King Sejong No BOTH)</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="3" t="inlineStr">
+      <c r="A38" s="4" t="inlineStr">
         <is>
           <t>Daejeon</t>
         </is>
       </c>
-      <c r="B38" s="3" t="inlineStr">
+      <c r="B38" s="4" t="inlineStr">
         <is>
           <t>NEONSAT-1A(67614)</t>
         </is>
       </c>
-      <c r="C38" s="3" t="inlineStr">
+      <c r="C38" s="4" t="inlineStr">
         <is>
           <t>Pass 14</t>
         </is>
       </c>
-      <c r="D38" s="3" t="inlineStr">
+      <c r="D38" s="4" t="inlineStr">
         <is>
           <t>2026-07-27 06:10:28</t>
         </is>
       </c>
-      <c r="E38" s="3" t="inlineStr">
+      <c r="E38" s="4" t="inlineStr">
         <is>
           <t>2026-07-27 06:18:23</t>
         </is>
       </c>
-      <c r="F38" s="3" t="n">
+      <c r="F38" s="4" t="n">
         <v>475.4</v>
       </c>
-      <c r="G38" s="3" t="n">
+      <c r="G38" s="4" t="n">
         <v>18.84</v>
       </c>
-      <c r="H38" s="3" t="inlineStr">
+      <c r="H38" s="4" t="inlineStr">
         <is>
           <t>Allocated</t>
         </is>
       </c>
-      <c r="I38" s="3" t="inlineStr">
+      <c r="I38" s="4" t="inlineStr">
         <is>
           <t>[7] 2차 Cal Maneuver (시나리오 등록 / Max logging / AOTM 다운)</t>
         </is>
@@ -2269,43 +2278,43 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="3" t="inlineStr">
+      <c r="A43" s="2" t="inlineStr">
         <is>
           <t>Svalbard</t>
         </is>
       </c>
-      <c r="B43" s="3" t="inlineStr">
+      <c r="B43" s="2" t="inlineStr">
         <is>
           <t>NEONSAT-1A(67614)</t>
         </is>
       </c>
-      <c r="C43" s="3" t="inlineStr">
+      <c r="C43" s="2" t="inlineStr">
         <is>
           <t>Pass 16</t>
         </is>
       </c>
-      <c r="D43" s="3" t="inlineStr">
+      <c r="D43" s="2" t="inlineStr">
         <is>
           <t>2026-07-27 10:46:50</t>
         </is>
       </c>
-      <c r="E43" s="3" t="inlineStr">
+      <c r="E43" s="2" t="inlineStr">
         <is>
           <t>2026-07-27 10:54:19</t>
         </is>
       </c>
-      <c r="F43" s="3" t="n">
+      <c r="F43" s="2" t="n">
         <v>448.7</v>
       </c>
-      <c r="G43" s="3" t="n">
+      <c r="G43" s="2" t="n">
         <v>15.22</v>
       </c>
-      <c r="H43" s="3" t="inlineStr">
-        <is>
-          <t>Bypassed</t>
-        </is>
-      </c>
-      <c r="I43" s="3" t="inlineStr">
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>Bypassed</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
         <is>
           <t>[3차 Cal Maneuver] Blocked (GS Svalbard No BOTH)</t>
         </is>

</xml_diff>